<commit_message>
3 DEC 2025 CLOSINGG
</commit_message>
<xml_diff>
--- a/NOVEMBER/NOVEMBER KITCHEN OUTSTANDING/NOVEMBER SURYA CIPTA NIAGA ABADI OUTSTANDING.xlsx
+++ b/NOVEMBER/NOVEMBER KITCHEN OUTSTANDING/NOVEMBER SURYA CIPTA NIAGA ABADI OUTSTANDING.xlsx
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>DATE</t>
   </si>
@@ -119,10 +119,16 @@
     <t>STRIPLOIN ICHI BROWN</t>
   </si>
   <si>
+    <t>PAID</t>
+  </si>
+  <si>
     <t>TOP SIDE BLACK ANGUS GF ONYX</t>
   </si>
   <si>
     <t>2511/FK-1864</t>
+  </si>
+  <si>
+    <t>UNPAID</t>
   </si>
   <si>
     <t>TOPSIDE WAGYU ONYX</t>
@@ -140,7 +146,7 @@
     <numFmt numFmtId="178" formatCode="[$-409]d\-mmm\-yyyy;@"/>
     <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,6 +177,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -315,7 +327,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -337,6 +349,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -753,76 +777,70 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -831,10 +849,10 @@
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -843,10 +861,10 @@
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -855,10 +873,10 @@
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -867,10 +885,10 @@
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -879,21 +897,24 @@
     <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -965,10 +986,16 @@
     <xf numFmtId="179" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1507,189 +1534,192 @@
   <dimension ref="A1:I13"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13.7142857142857" style="3" customWidth="1"/>
-    <col min="3" max="3" width="28.8571428571429" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.4285714285714" style="1" customWidth="1"/>
-    <col min="5" max="5" width="36.552380952381" style="1" customWidth="1"/>
-    <col min="6" max="7" width="18.7142857142857" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.8571428571429" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.4285714285714" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.14285714285714" style="1"/>
+    <col min="1" max="1" width="19" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7142857142857" style="2" customWidth="1"/>
+    <col min="3" max="3" width="28.8571428571429" customWidth="1"/>
+    <col min="4" max="4" width="25.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="36.552380952381" customWidth="1"/>
+    <col min="6" max="7" width="18.7142857142857" customWidth="1"/>
+    <col min="8" max="8" width="22.8571428571429" customWidth="1"/>
+    <col min="9" max="9" width="15.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="16" customHeight="1" spans="1:9">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="1" ht="16" customHeight="1" spans="1:9">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="55" customHeight="1" spans="1:9">
-      <c r="A2" s="7">
+    <row r="2" customFormat="1" ht="55" customHeight="1" spans="1:9">
+      <c r="A2" s="6">
         <v>45962</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="9">
         <v>11.79</v>
       </c>
-      <c r="E2" s="11" t="str">
+      <c r="E2" s="10" t="str">
         <f>_xlfn.DISPIMG("ID_B7457DA6CFC04C12B9163F9E9156146E",1)</f>
         <v>=DISPIMG("ID_B7457DA6CFC04C12B9163F9E9156146E",1)</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="11">
         <v>180000</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2" s="12">
         <f>D2*F2</f>
         <v>2122200</v>
       </c>
-      <c r="H2" s="13">
+      <c r="H2" s="12">
         <f>SUM(G2:G3)</f>
         <v>5277200</v>
       </c>
-      <c r="I2" s="27"/>
+      <c r="I2" s="26" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" s="1" customFormat="1" ht="55" customHeight="1" spans="1:9">
-      <c r="A3" s="14"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="10">
+    <row r="3" customFormat="1" ht="55" customHeight="1" spans="1:9">
+      <c r="A3" s="13"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="9">
         <v>12.62</v>
       </c>
-      <c r="E3" s="16"/>
-      <c r="F3" s="12">
+      <c r="E3" s="15"/>
+      <c r="F3" s="11">
         <v>250000</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3" s="12">
         <f>D3*F3</f>
         <v>3155000</v>
       </c>
-      <c r="H3" s="17"/>
-      <c r="I3" s="28"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="27"/>
     </row>
-    <row r="4" s="1" customFormat="1" ht="55" customHeight="1" spans="1:9">
-      <c r="A4" s="7">
+    <row r="4" customFormat="1" ht="55" customHeight="1" spans="1:9">
+      <c r="A4" s="6">
         <v>45976</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="9" t="s">
+      <c r="B4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>11.28</v>
       </c>
-      <c r="E4" s="18" t="str">
+      <c r="E4" s="17" t="str">
         <f>_xlfn.DISPIMG("ID_AD391E00A66A474F8756047855F2805B",1)</f>
         <v>=DISPIMG("ID_AD391E00A66A474F8756047855F2805B",1)</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="11">
         <v>180000</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="12">
         <f>D4*F4</f>
         <v>2030400</v>
       </c>
-      <c r="H4" s="13">
+      <c r="H4" s="12">
         <f>SUM(G4:G5)</f>
         <v>8140400</v>
       </c>
-      <c r="I4" s="27"/>
+      <c r="I4" s="28" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="55" customHeight="1" spans="1:9">
-      <c r="A5" s="14"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="10">
+    <row r="5" customFormat="1" ht="55" customHeight="1" spans="1:9">
+      <c r="A5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="9">
         <v>24.44</v>
       </c>
-      <c r="E5" s="19"/>
-      <c r="F5" s="12">
+      <c r="E5" s="18"/>
+      <c r="F5" s="11">
         <v>250000</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="12">
         <f>D5*F5</f>
         <v>6110000</v>
       </c>
-      <c r="H5" s="17"/>
-      <c r="I5" s="28"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="29"/>
     </row>
-    <row r="6" s="1" customFormat="1" ht="60" customHeight="1" spans="1:9">
-      <c r="A6" s="20" t="s">
+    <row r="6" customFormat="1" ht="23.25" spans="1:9">
+      <c r="A6" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="26">
-        <f>SUM(H2:H5)</f>
-        <v>13417600</v>
-      </c>
-      <c r="I6" s="26"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="25">
+        <f>SUM(H4)</f>
+        <v>8140400</v>
+      </c>
+      <c r="I6" s="25"/>
     </row>
-    <row r="7" s="1" customFormat="1" ht="60" customHeight="1" spans="1:2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
+    <row r="7" customFormat="1" ht="60" customHeight="1" spans="1:2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2"/>
     </row>
-    <row r="8" s="1" customFormat="1" ht="180" customHeight="1" spans="1:2">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
+    <row r="8" customFormat="1" ht="180" customHeight="1" spans="1:2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
     </row>
-    <row r="9" s="1" customFormat="1" spans="1:2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
+    <row r="9" customFormat="1" spans="1:2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
     </row>
-    <row r="10" s="1" customFormat="1" spans="1:2">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
+    <row r="10" customFormat="1" spans="1:2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="2"/>
     </row>
-    <row r="11" s="1" customFormat="1" spans="1:2">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
+    <row r="11" customFormat="1" spans="1:2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="2"/>
     </row>
-    <row r="12" s="1" customFormat="1" spans="1:2">
-      <c r="A12" s="2"/>
-      <c r="B12" s="3"/>
+    <row r="12" customFormat="1" spans="1:2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="2"/>
     </row>
-    <row r="13" s="1" customFormat="1" spans="1:2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
+    <row r="13" customFormat="1" spans="1:2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>

<commit_message>
15 December 2025 16.17 PM
</commit_message>
<xml_diff>
--- a/NOVEMBER/NOVEMBER KITCHEN OUTSTANDING/NOVEMBER SURYA CIPTA NIAGA ABADI OUTSTANDING.xlsx
+++ b/NOVEMBER/NOVEMBER KITCHEN OUTSTANDING/NOVEMBER SURYA CIPTA NIAGA ABADI OUTSTANDING.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7500"/>
+    <workbookView windowHeight="17000"/>
   </bookViews>
   <sheets>
     <sheet name="SURYA CIPTA NIAGA ABADI (BEEF)" sheetId="1" r:id="rId1"/>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>DATE</t>
   </si>
@@ -128,9 +128,6 @@
     <t>2511/FK-1864</t>
   </si>
   <si>
-    <t>UNPAID</t>
-  </si>
-  <si>
     <t>TOPSIDE WAGYU ONYX</t>
   </si>
 </sst>
@@ -139,12 +136,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="6">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="[$-409]d\-mmm\-yyyy;@"/>
-    <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="180" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+    <numFmt numFmtId="181" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -327,7 +324,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -355,12 +352,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -599,24 +590,26 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -627,17 +620,6 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -654,6 +636,15 @@
       <top style="thin">
         <color auto="1"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -765,16 +756,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -783,7 +774,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -807,16 +798,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -825,99 +816,99 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -926,76 +917,70 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1531,17 +1516,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelRow="7"/>
   <cols>
     <col min="1" max="1" width="19" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7142857142857" style="2" customWidth="1"/>
-    <col min="3" max="3" width="28.8571428571429" customWidth="1"/>
-    <col min="4" max="4" width="25.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="36.552380952381" customWidth="1"/>
-    <col min="6" max="7" width="18.7142857142857" customWidth="1"/>
-    <col min="8" max="8" width="22.8571428571429" customWidth="1"/>
-    <col min="9" max="9" width="15.4285714285714" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="28.859375" customWidth="1"/>
+    <col min="4" max="4" width="25.4296875" customWidth="1"/>
+    <col min="5" max="5" width="36.5546875" customWidth="1"/>
+    <col min="6" max="7" width="18.7109375" customWidth="1"/>
+    <col min="8" max="8" width="22.859375" customWidth="1"/>
+    <col min="9" max="9" width="15.4296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" ht="16" customHeight="1" spans="1:9">
@@ -1586,18 +1571,18 @@
       <c r="D2" s="9">
         <v>11.79</v>
       </c>
-      <c r="E2" s="10" t="str">
+      <c r="E2" s="15" t="str">
         <f>_xlfn.DISPIMG("ID_B7457DA6CFC04C12B9163F9E9156146E",1)</f>
         <v>=DISPIMG("ID_B7457DA6CFC04C12B9163F9E9156146E",1)</v>
       </c>
-      <c r="F2" s="11">
+      <c r="F2" s="16">
         <v>180000</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="17">
         <f>D2*F2</f>
         <v>2122200</v>
       </c>
-      <c r="H2" s="12">
+      <c r="H2" s="17">
         <f>SUM(G2:G3)</f>
         <v>5277200</v>
       </c>
@@ -1606,23 +1591,23 @@
       </c>
     </row>
     <row r="3" customFormat="1" ht="55" customHeight="1" spans="1:9">
-      <c r="A3" s="13"/>
-      <c r="B3" s="14"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="9">
         <v>12.62</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="11">
+      <c r="E3" s="18"/>
+      <c r="F3" s="16">
         <v>250000</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="17">
         <f>D3*F3</f>
         <v>3155000</v>
       </c>
-      <c r="H3" s="16"/>
+      <c r="H3" s="19"/>
       <c r="I3" s="27"/>
     </row>
     <row r="4" customFormat="1" ht="55" customHeight="1" spans="1:9">
@@ -1638,52 +1623,52 @@
       <c r="D4" s="9">
         <v>11.28</v>
       </c>
-      <c r="E4" s="17" t="str">
+      <c r="E4" s="20" t="str">
         <f>_xlfn.DISPIMG("ID_AD391E00A66A474F8756047855F2805B",1)</f>
         <v>=DISPIMG("ID_AD391E00A66A474F8756047855F2805B",1)</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="16">
         <v>180000</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="17">
         <f>D4*F4</f>
         <v>2030400</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="17">
         <f>SUM(G4:G5)</f>
         <v>8140400</v>
       </c>
-      <c r="I4" s="28" t="s">
-        <v>14</v>
+      <c r="I4" s="26" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="1" ht="55" customHeight="1" spans="1:9">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" s="9">
         <v>24.44</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="11">
+      <c r="E5" s="21"/>
+      <c r="F5" s="16">
         <v>250000</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="17">
         <f>D5*F5</f>
         <v>6110000</v>
       </c>
-      <c r="H5" s="16"/>
-      <c r="I5" s="29"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="27"/>
     </row>
-    <row r="6" customFormat="1" ht="23.25" spans="1:9">
-      <c r="A6" s="19" t="s">
+    <row r="6" customFormat="1" ht="26" spans="1:9">
+      <c r="A6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="13"/>
       <c r="E6" s="22"/>
       <c r="F6" s="23"/>
       <c r="G6" s="24"/>
@@ -1693,34 +1678,8 @@
       </c>
       <c r="I6" s="25"/>
     </row>
-    <row r="7" customFormat="1" ht="60" customHeight="1" spans="1:2">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" customFormat="1" ht="180" customHeight="1" spans="1:2">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" customFormat="1" spans="1:2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" customFormat="1" spans="1:2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" customFormat="1" spans="1:2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" customFormat="1" spans="1:2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" customFormat="1" spans="1:2">
-      <c r="A13" s="1"/>
-      <c r="B13" s="2"/>
-    </row>
+    <row r="7" ht="60" customHeight="1"/>
+    <row r="8" ht="180" customHeight="1"/>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A6:C6"/>

</xml_diff>